<commit_message>
Cập nhật hệ thống tra cứu theo STT
</commit_message>
<xml_diff>
--- a/tools/Danh mục.xlsx
+++ b/tools/Danh mục.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="112">
   <si>
     <t>Phụ lục 
 DANH MỤC CÁC HIỆN VẬT TRONG NHÀ TRUYỀN THỐNG
@@ -1085,7 +1085,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1116,6 +1116,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1129,13 +1135,22 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
@@ -1674,7 +1689,7 @@
   <dimension ref="A1:E50"/>
   <sheetFormatPr defaultColWidth="46.3636363636364" defaultRowHeight="14.5" outlineLevelCol="4"/>
   <cols>
-    <col min="1" max="1" width="5.54545454545455" style="1" customWidth="1"/>
+    <col min="1" max="1" width="6.88181818181818" style="1" customWidth="1"/>
     <col min="2" max="2" width="20.8181818181818" style="1" customWidth="1"/>
     <col min="3" max="3" width="30.4545454545455" style="1" customWidth="1"/>
     <col min="4" max="4" width="32.4545454545455" style="1" customWidth="1"/>
@@ -1947,7 +1962,7 @@
       <c r="D19" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E19" s="7" t="s">
+      <c r="E19" s="10" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1960,9 +1975,9 @@
       <c r="D20" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" ht="18.75" spans="1:5">
+      <c r="E20" s="11"/>
+    </row>
+    <row r="21" ht="36.75" spans="1:5">
       <c r="A21" s="7">
         <v>13</v>
       </c>
@@ -1975,410 +1990,420 @@
       <c r="D21" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="E21" s="7"/>
+      <c r="E21" s="7" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="22" ht="17.25" spans="1:5">
-      <c r="A22" s="10">
-        <v>1</v>
-      </c>
-      <c r="B22" s="10" t="s">
+      <c r="A22" s="12">
+        <v>14</v>
+      </c>
+      <c r="B22" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="C22" s="13" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="E22" s="12" t="s">
+      <c r="E22" s="14" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="23" ht="17.25" spans="1:5">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10" t="s">
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="12"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" ht="33.75" spans="1:5">
-      <c r="A24" s="10">
-        <v>2</v>
-      </c>
-      <c r="B24" s="10" t="s">
+      <c r="A24" s="12">
+        <v>15</v>
+      </c>
+      <c r="B24" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" s="12" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="13" t="s">
+      <c r="E24" s="15" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="25" ht="33.75" spans="1:5">
-      <c r="A25" s="10">
-        <v>3</v>
-      </c>
-      <c r="B25" s="10" t="s">
+      <c r="A25" s="12">
+        <v>16</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="13" t="s">
+      <c r="E25" s="15" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="26" ht="17.25" spans="1:5">
-      <c r="A26" s="10">
-        <v>4</v>
-      </c>
-      <c r="B26" s="10" t="s">
+    <row r="26" ht="49.5" spans="1:5">
+      <c r="A26" s="12">
+        <v>17</v>
+      </c>
+      <c r="B26" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="E26" s="16" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="27" ht="29" customHeight="1" spans="1:5">
-      <c r="A27" s="10">
-        <v>5</v>
-      </c>
-      <c r="B27" s="10" t="s">
+      <c r="A27" s="12">
+        <v>18</v>
+      </c>
+      <c r="B27" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E27" s="14"/>
+      <c r="E27" s="16" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1" spans="1:5">
-      <c r="A28" s="10">
-        <v>6</v>
-      </c>
-      <c r="B28" s="15" t="s">
+      <c r="A28" s="12">
+        <v>19</v>
+      </c>
+      <c r="B28" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E28" s="14" t="s">
+      <c r="E28" s="18" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1" spans="1:5">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10" t="s">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10" t="s">
+      <c r="C29" s="12"/>
+      <c r="D29" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="E29" s="14"/>
+      <c r="E29" s="18"/>
     </row>
     <row r="30" ht="18" customHeight="1" spans="1:5">
-      <c r="A30" s="10">
-        <v>7</v>
-      </c>
-      <c r="B30" s="15" t="s">
+      <c r="A30" s="12">
+        <v>20</v>
+      </c>
+      <c r="B30" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D30" s="10"/>
-      <c r="E30" s="13"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="15"/>
     </row>
     <row r="31" ht="18" customHeight="1" spans="1:5">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10" t="s">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="13"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="15"/>
     </row>
     <row r="32" ht="18" customHeight="1" spans="1:5">
-      <c r="A32" s="10">
+      <c r="A32" s="12">
+        <v>21</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="D32" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E32" s="15"/>
+    </row>
+    <row r="33" ht="18" customHeight="1" spans="1:5">
+      <c r="A33" s="12">
+        <v>22</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" ht="17.25" spans="1:5">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="B32" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C32" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="D32" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E32" s="13"/>
-    </row>
-    <row r="33" ht="18" customHeight="1" spans="1:5">
-      <c r="A33" s="10">
-        <v>9</v>
-      </c>
-      <c r="B33" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>76</v>
-      </c>
-      <c r="E33" s="14" t="s">
+      <c r="E34" s="21"/>
+    </row>
+    <row r="35" ht="33.75" spans="1:5">
+      <c r="A35" s="12">
+        <v>23</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E35" s="16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="34" ht="17.25" spans="1:5">
-      <c r="A34" s="10"/>
-      <c r="B34" s="10"/>
-      <c r="C34" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D34" s="10" t="s">
+    <row r="36" ht="33.75" spans="1:5">
+      <c r="A36" s="12">
+        <v>24</v>
+      </c>
+      <c r="B36" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D36" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="E34" s="14"/>
-    </row>
-    <row r="35" ht="17.25" spans="1:5">
-      <c r="A35" s="10">
-        <v>10</v>
-      </c>
-      <c r="B35" s="10" t="s">
+      <c r="E36" s="16" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="37" ht="16.5" spans="1:5">
+      <c r="A37" s="12">
+        <v>25</v>
+      </c>
+      <c r="B37" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="C35" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="D35" s="10" t="s">
+      <c r="C37" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E35" s="14"/>
-    </row>
-    <row r="36" ht="17.25" spans="1:5">
-      <c r="A36" s="10">
-        <v>11</v>
-      </c>
-      <c r="B36" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C36" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="D36" s="10" t="s">
-        <v>8</v>
-      </c>
-      <c r="E36" s="14"/>
-    </row>
-    <row r="37" ht="17.25" spans="1:5">
-      <c r="A37" s="10">
-        <v>12</v>
-      </c>
-      <c r="B37" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="C37" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="E37" s="14"/>
+      <c r="E37" s="20" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="38" ht="17.25" spans="1:5">
-      <c r="A38" s="10"/>
-      <c r="B38" s="10"/>
-      <c r="C38" s="10"/>
-      <c r="D38" s="10" t="s">
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="E38" s="14"/>
+      <c r="E38" s="21"/>
     </row>
     <row r="39" ht="33.75" spans="1:5">
-      <c r="A39" s="10">
-        <v>13</v>
-      </c>
-      <c r="B39" s="10" t="s">
+      <c r="A39" s="12">
+        <v>26</v>
+      </c>
+      <c r="B39" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="10"/>
-      <c r="E39" s="14" t="s">
+      <c r="D39" s="12"/>
+      <c r="E39" s="18" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="40" ht="33.75" spans="1:5">
-      <c r="A40" s="10">
-        <v>14</v>
-      </c>
-      <c r="B40" s="10" t="s">
+      <c r="A40" s="12">
+        <v>27</v>
+      </c>
+      <c r="B40" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="D40" s="10"/>
-      <c r="E40" s="14" t="s">
+      <c r="D40" s="12"/>
+      <c r="E40" s="18" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="41" ht="33.75" spans="1:5">
-      <c r="A41" s="10">
-        <v>15</v>
-      </c>
-      <c r="B41" s="10" t="s">
+      <c r="A41" s="12">
+        <v>28</v>
+      </c>
+      <c r="B41" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="15" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="42" ht="33.75" spans="1:5">
-      <c r="A42" s="10">
-        <v>16</v>
-      </c>
-      <c r="B42" s="10" t="s">
+      <c r="A42" s="12">
+        <v>29</v>
+      </c>
+      <c r="B42" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="16"/>
-      <c r="D42" s="10"/>
-      <c r="E42" s="14" t="s">
+      <c r="C42" s="19"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="18" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="43" ht="50.25" spans="1:5">
-      <c r="A43" s="10">
-        <v>17</v>
-      </c>
-      <c r="B43" s="10" t="s">
+      <c r="A43" s="12">
+        <v>30</v>
+      </c>
+      <c r="B43" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="C43" s="17"/>
-      <c r="D43" s="18"/>
-      <c r="E43" s="19" t="s">
+      <c r="C43" s="22"/>
+      <c r="D43" s="23"/>
+      <c r="E43" s="24" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="44" ht="50.25" spans="1:5">
-      <c r="A44" s="10">
-        <v>18</v>
-      </c>
-      <c r="B44" s="10" t="s">
+      <c r="A44" s="12">
+        <v>31</v>
+      </c>
+      <c r="B44" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="16"/>
-      <c r="D44" s="10"/>
-      <c r="E44" s="14" t="s">
+      <c r="C44" s="19"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="18" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="45" ht="50.25" spans="1:5">
-      <c r="A45" s="10">
-        <v>19</v>
-      </c>
-      <c r="B45" s="10" t="s">
+      <c r="A45" s="12">
+        <v>32</v>
+      </c>
+      <c r="B45" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="C45" s="16"/>
-      <c r="D45" s="10"/>
-      <c r="E45" s="14" t="s">
+      <c r="C45" s="19"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="18" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="46" ht="50.25" spans="1:5">
-      <c r="A46" s="10">
-        <v>20</v>
-      </c>
-      <c r="B46" s="10" t="s">
+      <c r="A46" s="12">
+        <v>33</v>
+      </c>
+      <c r="B46" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="16"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="14" t="s">
+      <c r="C46" s="19"/>
+      <c r="D46" s="12"/>
+      <c r="E46" s="18" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="47" ht="50.25" spans="1:5">
-      <c r="A47" s="10">
-        <v>21</v>
-      </c>
-      <c r="B47" s="10" t="s">
+      <c r="A47" s="12">
+        <v>34</v>
+      </c>
+      <c r="B47" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="16"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="14" t="s">
+      <c r="C47" s="19"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="18" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="48" ht="33.75" spans="1:5">
-      <c r="A48" s="10">
-        <v>22</v>
-      </c>
-      <c r="B48" s="10" t="s">
+      <c r="A48" s="12">
+        <v>35</v>
+      </c>
+      <c r="B48" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="C48" s="16"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="14" t="s">
+      <c r="C48" s="19"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="18" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="49" ht="50.25" spans="1:5">
-      <c r="A49" s="10">
-        <v>23</v>
-      </c>
-      <c r="B49" s="10" t="s">
+      <c r="A49" s="12">
+        <v>36</v>
+      </c>
+      <c r="B49" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="C49" s="16"/>
-      <c r="D49" s="10"/>
-      <c r="E49" s="14" t="s">
+      <c r="C49" s="19"/>
+      <c r="D49" s="12"/>
+      <c r="E49" s="18" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="50" ht="33.75" spans="1:5">
-      <c r="A50" s="10">
-        <v>24</v>
-      </c>
-      <c r="B50" s="10" t="s">
+      <c r="A50" s="12">
+        <v>37</v>
+      </c>
+      <c r="B50" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="C50" s="16"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="14" t="s">
+      <c r="C50" s="19"/>
+      <c r="D50" s="12"/>
+      <c r="E50" s="18" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2413,12 +2438,12 @@
     <mergeCell ref="E6:E7"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="E17:E18"/>
-    <mergeCell ref="E19:E21"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="E22:E23"/>
-    <mergeCell ref="E26:E27"/>
     <mergeCell ref="E28:E29"/>
     <mergeCell ref="E30:E31"/>
-    <mergeCell ref="E33:E38"/>
+    <mergeCell ref="E33:E34"/>
+    <mergeCell ref="E37:E38"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>